<commit_message>
aktualizacja i przeróbka 164
</commit_message>
<xml_diff>
--- a/164/data/164_liczba-zmian-kadrowych-w-spolkach-skarbu-panstwa.xlsx
+++ b/164/data/164_liczba-zmian-kadrowych-w-spolkach-skarbu-panstwa.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="198">
   <si>
     <t xml:space="preserve">Case name</t>
   </si>
@@ -693,6 +693,41 @@
   </si>
   <si>
     <t xml:space="preserve">w okresach podanych we wniosku Spółka ani nie rozpoczęła współpracy z osobami zatrudnianymi na stanowiskach – jak we wniosku – ani nie zakończyła współpracy z osobami na takich stanowiskach. W  Spółce w tych okresach nie funkcjonowały takie stanowiska.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liczba zmian kadrowych w spółkach skarbu państwa #10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">liczba-zmian-kadrowych-w-spolkach-skarbu-panstwa-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://fedrowanie.siecobywatelska.pl/sprawy/liczba-zmian-kadrowych-w-spolkach-skarbu-panstwa-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Polskie Elektrownie Jądrowe Sp. z o.o.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sekretariat@ppej.pl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://fedrowanie.siecobywatelska.pl/listy/493660</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-15 08:55:51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Okresy|Nawiązanie współpracy|Zakończenie współpracy
+od 1 maja 2015 r. do 31 października 2015 r.|5|0
+od 1 listopada 2015 r. do 30 kwietnia 2016 r.|1|2
+od 1 listopada 2019 r. do 30 kwietnia 2020 r.|0|2
+od 1 maja 2023 r. do 31 października 2023 r.|9|2
+od 1 listopada 2023 r. do 30 kwietnia 2024 r.|6|5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"2015-05-01_2015-10-31": 5, "2015-11-01_2016-04-30": 1, "2019-11-01_2020-04-30": 0, "2023-05-01_2023-10-31": 9, "2023-11-01_2024-04-30": 6}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"2015-05-01_2015-10-31": 0, "2015-11-01_2016-04-30": 2, "2019-11-01_2020-04-30": 2, "2023-05-01_2023-10-31": 2, "2023-11-01_2024-04-30": 5}</t>
   </si>
 </sst>
 </file>
@@ -1003,7 +1038,7 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="29.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16381" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16381" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="38.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2562,6 +2597,142 @@
       </c>
       <c r="V23" s="1" t="s">
         <v>148</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="162.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B24" s="1" t="n">
+        <v>125092</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="F24" s="1" t="n">
+        <v>8289</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="L24" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="M24" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="N24" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="O24" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="P24" s="1" t="n">
+        <v>493660</v>
+      </c>
+      <c r="Q24" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="R24" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="S24" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="T24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U24" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="V24" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="162.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B25" s="1" t="n">
+        <v>125092</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="F25" s="1" t="n">
+        <v>8289</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="L25" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="M25" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="N25" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="O25" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="P25" s="1" t="n">
+        <v>493660</v>
+      </c>
+      <c r="Q25" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="R25" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="S25" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="T25" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="U25" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="V25" s="1" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="1048535" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>